<commit_message>
chore: sync Nova upm-release-2026.08.14-01
</commit_message>
<xml_diff>
--- a/Assets/Samples/AIHelpDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
+++ b/Assets/Samples/AIHelpDemo/Excels/Networks/HostKeys/NetworkHostKeys.xlsx
@@ -1191,7 +1191,11 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="E2" s="5" t="n"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>FallbackValue</t>
+        </is>
+      </c>
       <c r="F2" s="5" t="n"/>
       <c r="G2" s="5" t="n"/>
       <c r="H2" s="5" t="n"/>
@@ -1233,7 +1237,11 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
@@ -1272,7 +1280,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>主域名</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>备用域名</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1306,11 @@
           <t>https://t-solo-api-game.ahameet.com</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://t-solo-api-game.ahameet.com</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
@@ -1331,7 +1348,11 @@
           <t>https://solotopia.aihelp.net</t>
         </is>
       </c>
-      <c r="E6" s="3" t="n"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://solotopia.aihelp.net</t>
+        </is>
+      </c>
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
@@ -1364,6 +1385,11 @@
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://report.lolipopmobi.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://report.lolipopmobi.com</t>
         </is>
@@ -1486,7 +1512,11 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="E2" s="5" t="n"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>FallbackValue</t>
+        </is>
+      </c>
       <c r="F2" s="5" t="n"/>
       <c r="G2" s="5" t="n"/>
       <c r="H2" s="5" t="n"/>
@@ -1528,7 +1558,11 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
@@ -1567,7 +1601,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>主域名</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>备用域名</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1627,11 @@
           <t>https://t-solo-api-game.ahameet.com</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://t-solo-api-game.ahameet.com</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
@@ -1626,7 +1669,11 @@
           <t>https://solotopia.aihelp.net</t>
         </is>
       </c>
-      <c r="E6" s="3" t="n"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://solotopia.aihelp.net</t>
+        </is>
+      </c>
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
@@ -1659,6 +1706,11 @@
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://report.lolipopmobi.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://report.lolipopmobi.com</t>
         </is>

</xml_diff>